<commit_message>
data OB fixed DCH 3 estaciones actualizada
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH/Carga_on_board_fixed_3estaciones/elmo_data.xlsx
+++ b/data/Escenarios_DCH/Carga_on_board_fixed_3estaciones/elmo_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_DCH\Carga_on_board_fixed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_DCH\Carga_on_board_fixed_3estaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7217129E-A84F-411C-ABCD-45F0FE60DB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5699DCF9-2E19-4A0E-B0B6-CBF4E521D9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -3446,19 +3446,19 @@
         <v>380</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>215756</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="E3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>5000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3469,19 +3469,19 @@
         <v>388</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>215756</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="E4">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>5000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3492,19 +3492,19 @@
         <v>389</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>215756</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="E5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>5000</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>